<commit_message>
Update comparison logic, UI config, tests, and sample data
</commit_message>
<xml_diff>
--- a/sample_data/GPVDS - Copy.xlsx
+++ b/sample_data/GPVDS - Copy.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ItemName</t>
+          <t>Drug Code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -435,6 +435,11 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>StockQty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expiry Date</t>
         </is>
       </c>
     </row>
@@ -454,8 +459,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>40</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>04-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -474,8 +486,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>60</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>06-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -494,8 +513,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>30</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>09-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -514,8 +540,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>45</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -534,8 +567,15 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>20</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>03-01-2027</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -554,8 +594,15 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>40</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>04-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -574,8 +621,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>20</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>06-01-2026</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -594,8 +648,15 @@
           <t>Delhi</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>25</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>09-01-2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>